<commit_message>
docs(audio_cinematics): Entscheidung 20-B (volle 60 s + 15 s Übergang), C20-Reprise mit 8 Zeilen, C15/C16 freigegeben mit vorläufigen Zeitcodes
</commit_message>
<xml_diff>
--- a/docs/audio_cinematics/genesis_sprachzeilen_C00-C21.xlsx
+++ b/docs/audio_cinematics/genesis_sprachzeilen_C00-C21.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$S$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$S$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S196"/>
+  <dimension ref="A1:S201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9950,12 +9950,22 @@
           <t>00:01:30:00</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>00:01:04:00</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>00:01:05:17</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>1.7</v>
+      </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -9990,7 +10000,7 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01); bedingt</t>
+          <t>Zeitcode vorläufig/geschätzt; bedingt</t>
         </is>
       </c>
       <c r="S107" t="inlineStr"/>
@@ -10031,12 +10041,22 @@
           <t>00:02:10:00</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>00:01:31:00</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>00:01:34:00</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>3</v>
+      </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -10071,7 +10091,7 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S108" t="inlineStr"/>
@@ -10112,12 +10132,22 @@
           <t>00:02:10:00</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>00:01:36:02</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>00:01:40:00</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>3.9</v>
+      </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -10148,7 +10178,7 @@
       </c>
       <c r="R109" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S109" t="inlineStr"/>
@@ -10189,12 +10219,22 @@
           <t>00:00:38:00</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>00:00:01:00</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>00:00:04:00</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>3</v>
+      </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -10225,7 +10265,7 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S110" t="inlineStr"/>
@@ -10266,12 +10306,22 @@
           <t>00:00:38:00</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>00:00:06:02</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>00:00:11:07</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>5.2</v>
+      </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -10302,7 +10352,7 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S111" t="inlineStr"/>
@@ -10343,12 +10393,22 @@
           <t>00:01:18:00</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>00:00:39:00</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>00:00:41:02</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>2.1</v>
+      </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -10383,7 +10443,7 @@
       </c>
       <c r="R112" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01); bedingt</t>
+          <t>Zeitcode vorläufig/geschätzt; bedingt</t>
         </is>
       </c>
       <c r="S112" t="inlineStr"/>
@@ -10424,12 +10484,22 @@
           <t>00:01:18:00</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>00:00:41:17</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>00:00:45:02</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>3.4</v>
+      </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -10460,7 +10530,7 @@
       </c>
       <c r="R113" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S113" t="inlineStr"/>
@@ -10501,12 +10571,22 @@
           <t>00:02:18:00</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>00:01:19:00</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>00:01:21:02</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>2.1</v>
+      </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -10537,7 +10617,7 @@
       </c>
       <c r="R114" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S114" t="inlineStr"/>
@@ -10578,12 +10658,22 @@
           <t>00:02:18:00</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>00:01:23:05</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>00:01:25:07</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>2.1</v>
+      </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -10618,7 +10708,7 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S115" t="inlineStr"/>
@@ -10659,12 +10749,22 @@
           <t>00:03:33:00</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>00:02:19:00</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>00:02:22:00</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>3</v>
+      </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -10695,7 +10795,7 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S116" t="inlineStr"/>
@@ -10736,12 +10836,22 @@
           <t>00:03:33:00</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>00:02:22:14</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>00:02:24:07</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>1.7</v>
+      </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -10772,7 +10882,7 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S117" t="inlineStr"/>
@@ -10813,12 +10923,22 @@
           <t>00:03:33:00</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>00:02:24:22</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>00:02:27:22</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
+        <v>3</v>
+      </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -10849,7 +10969,7 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S118" t="inlineStr"/>
@@ -10890,12 +11010,22 @@
           <t>00:03:33:00</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>00:02:28:12</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>00:02:32:19</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>4.3</v>
+      </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -10926,7 +11056,7 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S119" t="inlineStr"/>
@@ -10967,12 +11097,22 @@
           <t>00:04:30:00</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>00:03:34:00</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>00:03:37:22</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>3.9</v>
+      </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -11003,7 +11143,7 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S120" t="inlineStr"/>
@@ -11044,12 +11184,22 @@
           <t>00:04:30:00</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>00:03:40:00</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>00:03:43:00</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>3</v>
+      </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>zurückgestellt, Kanon-Entscheidung CON33-01 offen</t>
+          <t>vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -11080,7 +11230,7 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>zurückgestellt (CON33-01)</t>
+          <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
       <c r="S121" t="inlineStr"/>
@@ -14876,7 +15026,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>20-B (Shot-Bereich 01:00–02:15)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -14896,12 +15046,12 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>00:01:01:00</t>
+          <t>00:01:26:12</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>00:01:04:10</t>
+          <t>00:01:29:22</t>
         </is>
       </c>
       <c r="J165" t="n">
@@ -14909,7 +15059,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -14935,12 +15085,12 @@
       <c r="P165" t="inlineStr"/>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>636</t>
+          <t>81</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_001, Zeile 81)</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_001, Zeile 81); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S165" t="inlineStr"/>
@@ -14963,7 +15113,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>20-B (Shot-Bereich 01:00–02:15)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -14983,12 +15133,12 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>00:01:05:00</t>
+          <t>00:01:30:12</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>00:01:08:22</t>
+          <t>00:01:34:10</t>
         </is>
       </c>
       <c r="J166" t="n">
@@ -14996,7 +15146,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -15019,15 +15169,19 @@
           <t>Ich weiß, dass du vieles anders machen wolltest.</t>
         </is>
       </c>
-      <c r="P166" t="inlineStr"/>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>sucht nicht nach einer beruhigenden Lüge</t>
+        </is>
+      </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>637</t>
+          <t>82</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_002, Zeile 82)</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_002, Zeile 82); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S166" t="inlineStr"/>
@@ -15050,7 +15204,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>20-B (Shot-Bereich 01:00–02:15)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -15070,25 +15224,25 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>00:01:09:12</t>
+          <t>00:01:35:00</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>00:01:15:14</t>
+          <t>00:01:38:22</t>
         </is>
       </c>
       <c r="J167" t="n">
-        <v>6.1</v>
+        <v>3.9</v>
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>TOCHTER</t>
+          <t>MANN, AUS C00 (ORIGINAL-O-TON)</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
@@ -15103,21 +15257,25 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>Manche Dinge bleiben bei den Menschen. Auch wenn man es selbst nie erfährt.</t>
+          <t>Es gibt so viel, das ich nie …</t>
         </is>
       </c>
       <c r="P167" t="inlineStr"/>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>638</t>
+          <t>83</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_006, Zeile 86)</t>
-        </is>
-      </c>
-      <c r="S167" t="inlineStr"/>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_003, Zeile 83); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>„so viel, das ich nie …“: nach „viel“ verlangt die Standardsprache „was“ (so viel, was …). Mögliche Absicht der Sprechweise – nicht geändert.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -15137,45 +15295,45 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>20-C (Shot-Bereich 02:15–03:35)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>20-C</t>
+          <t>20-B</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
+          <t>00:01:00:00</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
           <t>00:02:15:00</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>00:03:35:00</t>
-        </is>
-      </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>00:02:16:00</t>
+          <t>00:01:39:12</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>00:02:18:14</t>
+          <t>00:01:40:19</t>
         </is>
       </c>
       <c r="J168" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>TOCHTER, AUS C00 (ORIGINAL-O-TON)</t>
         </is>
       </c>
       <c r="M168" t="inlineStr">
@@ -15190,18 +15348,18 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>Das … war mein Leben?</t>
+          <t>Ich weiß.</t>
         </is>
       </c>
       <c r="P168" t="inlineStr"/>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>84</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_004, Zeile 84); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S168" t="inlineStr"/>
@@ -15224,45 +15382,45 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>20-C (Shot-Bereich 02:15–03:35)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>20-C</t>
+          <t>20-B</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
+          <t>00:01:00:00</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
           <t>00:02:15:00</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>00:03:35:00</t>
-        </is>
-      </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>00:02:19:05</t>
+          <t>00:01:41:10</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>00:02:23:22</t>
+          <t>00:01:44:10</t>
         </is>
       </c>
       <c r="J169" t="n">
-        <v>4.7</v>
+        <v>3</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>MANN, AUS C00 (ORIGINAL-O-TON)</t>
         </is>
       </c>
       <c r="M169" t="inlineStr">
@@ -15277,18 +15435,18 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>Ein Leben vor den deinen. Dasselbe Echo. Nicht derselbe Mensch.</t>
+          <t>Und was, wenn nichts davon bleibt?</t>
         </is>
       </c>
       <c r="P169" t="inlineStr"/>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>85</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_005, Zeile 85); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S169" t="inlineStr"/>
@@ -15311,45 +15469,45 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>20-C (Shot-Bereich 02:15–03:35)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>20-C</t>
+          <t>20-B</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
+          <t>00:01:00:00</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
           <t>00:02:15:00</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>00:03:35:00</t>
-        </is>
-      </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>00:02:24:12</t>
+          <t>00:01:45:00</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>00:02:27:12</t>
+          <t>00:01:51:02</t>
         </is>
       </c>
       <c r="J170" t="n">
-        <v>3</v>
+        <v>6.1</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>TOCHTER, AUS C00 (ORIGINAL-O-TON)</t>
         </is>
       </c>
       <c r="M170" t="inlineStr">
@@ -15364,18 +15522,18 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>Aber ich erinnere mich nicht daran.</t>
+          <t>Manche Dinge bleiben bei den Menschen. Auch wenn man es selbst nie erfährt.</t>
         </is>
       </c>
       <c r="P170" t="inlineStr"/>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>86</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_006, Zeile 86); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S170" t="inlineStr"/>
@@ -15398,45 +15556,45 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>20-C (Shot-Bereich 02:15–03:35)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>20-C</t>
+          <t>20-B</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
+          <t>00:01:00:00</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
           <t>00:02:15:00</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>00:03:35:00</t>
-        </is>
-      </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>00:02:28:02</t>
+          <t>00:01:51:17</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>00:02:32:10</t>
+          <t>00:01:53:19</t>
         </is>
       </c>
       <c r="J171" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>MANN, AUS C00 (ORIGINAL-O-TON)</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
@@ -15451,18 +15609,18 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>Weil ein neues Leben ein eigenes Leben sein muss.</t>
+          <t>Das weiß ich nicht.</t>
         </is>
       </c>
       <c r="P171" t="inlineStr"/>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>645</t>
+          <t>87</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_007, Zeile 87); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S171" t="inlineStr"/>
@@ -15485,45 +15643,45 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>20-C (Shot-Bereich 02:15–03:35)</t>
+          <t>20-B (Shot-Bereich 01:00–02:15, Reprise 01:07:12–02:07:12)</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>20-C</t>
+          <t>20-B</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
+          <t>00:01:00:00</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
           <t>00:02:15:00</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>00:03:35:00</t>
-        </is>
-      </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>00:02:33:00</t>
+          <t>00:01:54:10</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>00:02:34:17</t>
+          <t>00:01:58:17</t>
         </is>
       </c>
       <c r="J172" t="n">
-        <v>1.7</v>
+        <v>4.3</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>vorläufig/geschätzt</t>
+          <t>vorläufig/geschätzt; folgt 1:1 aus C00 (+55,5 s)</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>TOCHTER, AUS C00 (ORIGINAL-O-TON)</t>
         </is>
       </c>
       <c r="M172" t="inlineStr">
@@ -15538,18 +15696,18 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>Und seine Tochter?</t>
+          <t>Du musst es jetzt nicht wissen. Ich bin hier.</t>
         </is>
       </c>
       <c r="P172" t="inlineStr"/>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>646</t>
+          <t>88</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>Zeitcode vorläufig/geschätzt</t>
+          <t>Zeitcode vorläufig/geschätzt; Reprise aus C00, Originalton – keine Neuaufnahme (Quelle VO_C00_008, Zeile 88); Entscheidung 23.10.2026: volle 60 s, alle 8 Zeilen</t>
         </is>
       </c>
       <c r="S172" t="inlineStr"/>
@@ -15592,16 +15750,16 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>00:02:35:07</t>
+          <t>00:02:16:00</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>00:02:40:22</t>
+          <t>00:02:18:14</t>
         </is>
       </c>
       <c r="J173" t="n">
-        <v>5.6</v>
+        <v>2.6</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -15610,7 +15768,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M173" t="inlineStr">
@@ -15625,13 +15783,13 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>Sie hatte ihr Leben. Ihre Geschichte ging weiter. Sie gehört nicht dir.</t>
+          <t>Das … war mein Leben?</t>
         </is>
       </c>
       <c r="P173" t="inlineStr"/>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>647</t>
+          <t>642</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
@@ -15659,36 +15817,36 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>20-D (Shot-Bereich 03:35–05:05)</t>
+          <t>20-C (Shot-Bereich 02:15–03:35)</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>20-D</t>
+          <t>20-C</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
+          <t>00:02:15:00</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
           <t>00:03:35:00</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>00:05:05:00</t>
-        </is>
-      </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>00:03:36:00</t>
+          <t>00:02:19:05</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>00:03:42:22</t>
+          <t>00:02:23:22</t>
         </is>
       </c>
       <c r="J174" t="n">
-        <v>6.9</v>
+        <v>4.7</v>
       </c>
       <c r="K174" t="inlineStr">
         <is>
@@ -15697,7 +15855,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M174" t="inlineStr">
@@ -15712,13 +15870,13 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>Er wollte wissen, ob er genug getan hatte. Und ich stelle mir die gleiche Frage.</t>
+          <t>Ein Leben vor den deinen. Dasselbe Echo. Nicht derselbe Mensch.</t>
         </is>
       </c>
       <c r="P174" t="inlineStr"/>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>651</t>
+          <t>643</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -15726,11 +15884,7 @@
           <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
-      <c r="S174" t="inlineStr">
-        <is>
-          <t>„die gleiche Frage“ – gemeint ist dieselbe Frage; stilistisch, in Alltagssprache akzeptiert.</t>
-        </is>
-      </c>
+      <c r="S174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -15750,36 +15904,36 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>20-D (Shot-Bereich 03:35–05:05)</t>
+          <t>20-C (Shot-Bereich 02:15–03:35)</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>20-D</t>
+          <t>20-C</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
+          <t>00:02:15:00</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
           <t>00:03:35:00</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>00:05:05:00</t>
-        </is>
-      </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>00:03:43:12</t>
+          <t>00:02:24:12</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>00:03:47:19</t>
+          <t>00:02:27:12</t>
         </is>
       </c>
       <c r="J175" t="n">
-        <v>4.3</v>
+        <v>3</v>
       </c>
       <c r="K175" t="inlineStr">
         <is>
@@ -15788,7 +15942,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
@@ -15803,13 +15957,13 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>Kein Leben lässt sich auf eine einzige Zahl reduzieren.</t>
+          <t>Aber ich erinnere mich nicht daran.</t>
         </is>
       </c>
       <c r="P175" t="inlineStr"/>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>644</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -15837,36 +15991,36 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>20-D (Shot-Bereich 03:35–05:05)</t>
+          <t>20-C (Shot-Bereich 02:15–03:35)</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>20-D</t>
+          <t>20-C</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
+          <t>00:02:15:00</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
           <t>00:03:35:00</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>00:05:05:00</t>
-        </is>
-      </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>00:03:48:10</t>
+          <t>00:02:28:02</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>00:03:51:00</t>
+          <t>00:02:32:10</t>
         </is>
       </c>
       <c r="J176" t="n">
-        <v>2.6</v>
+        <v>4.3</v>
       </c>
       <c r="K176" t="inlineStr">
         <is>
@@ -15875,7 +16029,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
@@ -15890,13 +16044,13 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>Aber ich habe andere verändert.</t>
+          <t>Weil ein neues Leben ein eigenes Leben sein muss.</t>
         </is>
       </c>
       <c r="P176" t="inlineStr"/>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>645</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -15924,36 +16078,36 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>20-D (Shot-Bereich 03:35–05:05)</t>
+          <t>20-C (Shot-Bereich 02:15–03:35)</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>20-D</t>
+          <t>20-C</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
+          <t>00:02:15:00</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
           <t>00:03:35:00</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>00:05:05:00</t>
-        </is>
-      </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>00:03:51:14</t>
+          <t>00:02:33:00</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>00:03:54:05</t>
+          <t>00:02:34:17</t>
         </is>
       </c>
       <c r="J177" t="n">
-        <v>2.6</v>
+        <v>1.7</v>
       </c>
       <c r="K177" t="inlineStr">
         <is>
@@ -15962,7 +16116,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
@@ -15977,13 +16131,13 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>Und sie haben dich verändert.</t>
+          <t>Und seine Tochter?</t>
         </is>
       </c>
       <c r="P177" t="inlineStr"/>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>654</t>
+          <t>646</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -16011,36 +16165,36 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>20-D (Shot-Bereich 03:35–05:05)</t>
+          <t>20-C (Shot-Bereich 02:15–03:35)</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>20-D</t>
+          <t>20-C</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
+          <t>00:02:15:00</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
           <t>00:03:35:00</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>00:05:05:00</t>
-        </is>
-      </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>00:03:54:19</t>
+          <t>00:02:35:07</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>00:03:59:02</t>
+          <t>00:02:40:22</t>
         </is>
       </c>
       <c r="J178" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="K178" t="inlineStr">
         <is>
@@ -16049,7 +16203,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
@@ -16064,13 +16218,13 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>Dann gibt es keinen Weg, alles richtig zu machen?</t>
+          <t>Sie hatte ihr Leben. Ihre Geschichte ging weiter. Sie gehört nicht dir.</t>
         </is>
       </c>
       <c r="P178" t="inlineStr"/>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>655</t>
+          <t>647</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
@@ -16118,16 +16272,16 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>00:03:59:17</t>
+          <t>00:03:36:00</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>00:04:02:17</t>
+          <t>00:03:42:22</t>
         </is>
       </c>
       <c r="J179" t="n">
-        <v>3</v>
+        <v>6.9</v>
       </c>
       <c r="K179" t="inlineStr">
         <is>
@@ -16136,7 +16290,7 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
@@ -16151,13 +16305,13 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>Es gibt Verantwortung. Keine vollständige Kontrolle.</t>
+          <t>Er wollte wissen, ob er genug getan hatte. Und ich stelle mir die gleiche Frage.</t>
         </is>
       </c>
       <c r="P179" t="inlineStr"/>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>656</t>
+          <t>651</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
@@ -16165,7 +16319,11 @@
           <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
-      <c r="S179" t="inlineStr"/>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>„die gleiche Frage“ – gemeint ist dieselbe Frage; stilistisch, in Alltagssprache akzeptiert.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -16185,36 +16343,36 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>20-E (Shot-Bereich 05:05–06:32)</t>
+          <t>20-D (Shot-Bereich 03:35–05:05)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>20-E</t>
+          <t>20-D</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
+          <t>00:03:35:00</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
           <t>00:05:05:00</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>00:06:32:00</t>
-        </is>
-      </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>00:05:06:00</t>
+          <t>00:03:43:12</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>00:05:09:00</t>
+          <t>00:03:47:19</t>
         </is>
       </c>
       <c r="J180" t="n">
-        <v>3</v>
+        <v>4.3</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
@@ -16223,7 +16381,7 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M180" t="inlineStr">
@@ -16238,13 +16396,13 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>Wer hat dann diese Welt erschaffen?</t>
+          <t>Kein Leben lässt sich auf eine einzige Zahl reduzieren.</t>
         </is>
       </c>
       <c r="P180" t="inlineStr"/>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>660</t>
+          <t>652</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -16272,36 +16430,36 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>20-E (Shot-Bereich 05:05–06:32)</t>
+          <t>20-D (Shot-Bereich 03:35–05:05)</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>20-E</t>
+          <t>20-D</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
+          <t>00:03:35:00</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
           <t>00:05:05:00</t>
         </is>
       </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>00:06:32:00</t>
-        </is>
-      </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>00:05:09:14</t>
+          <t>00:03:48:10</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>00:05:12:14</t>
+          <t>00:03:51:00</t>
         </is>
       </c>
       <c r="J181" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
@@ -16310,7 +16468,7 @@
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
@@ -16325,13 +16483,13 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>Den ersten Ursprung kennen wir nicht.</t>
+          <t>Aber ich habe andere verändert.</t>
         </is>
       </c>
       <c r="P181" t="inlineStr"/>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>661</t>
+          <t>653</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
@@ -16359,36 +16517,36 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>20-E (Shot-Bereich 05:05–06:32)</t>
+          <t>20-D (Shot-Bereich 03:35–05:05)</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>20-E</t>
+          <t>20-D</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
+          <t>00:03:35:00</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
           <t>00:05:05:00</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr">
-        <is>
-          <t>00:06:32:00</t>
-        </is>
-      </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>00:05:14:17</t>
+          <t>00:03:51:14</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>00:05:24:05</t>
+          <t>00:03:54:05</t>
         </is>
       </c>
       <c r="J182" t="n">
-        <v>9.5</v>
+        <v>2.6</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
@@ -16412,13 +16570,13 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>Aber die Welt, in der Menschen leben – ihre Häuser, Geschichten, Hoffnungen, ihre Wunden und ihre Möglichkeiten – formen sie miteinander.</t>
+          <t>Und sie haben dich verändert.</t>
         </is>
       </c>
       <c r="P182" t="inlineStr"/>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>663</t>
+          <t>654</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -16446,36 +16604,36 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>20-E (Shot-Bereich 05:05–06:32)</t>
+          <t>20-D (Shot-Bereich 03:35–05:05)</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>20-E</t>
+          <t>20-D</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
+          <t>00:03:35:00</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
           <t>00:05:05:00</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>00:06:32:00</t>
-        </is>
-      </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>00:05:24:19</t>
+          <t>00:03:54:19</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>00:05:26:02</t>
+          <t>00:03:59:02</t>
         </is>
       </c>
       <c r="J183" t="n">
-        <v>1.3</v>
+        <v>4.3</v>
       </c>
       <c r="K183" t="inlineStr">
         <is>
@@ -16499,13 +16657,13 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>Wir alle?</t>
+          <t>Dann gibt es keinen Weg, alles richtig zu machen?</t>
         </is>
       </c>
       <c r="P183" t="inlineStr"/>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>664</t>
+          <t>655</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
@@ -16533,36 +16691,36 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>20-E (Shot-Bereich 05:05–06:32)</t>
+          <t>20-D (Shot-Bereich 03:35–05:05)</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>20-E</t>
+          <t>20-D</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
+          <t>00:03:35:00</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
           <t>00:05:05:00</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>00:06:32:00</t>
-        </is>
-      </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>00:05:26:17</t>
+          <t>00:03:59:17</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>00:05:33:14</t>
+          <t>00:04:02:17</t>
         </is>
       </c>
       <c r="J184" t="n">
-        <v>6.9</v>
+        <v>3</v>
       </c>
       <c r="K184" t="inlineStr">
         <is>
@@ -16586,13 +16744,13 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>Mit jedem Leben. Mit dem, was wir tun. Und mit dem, was wir anderen ermöglichen.</t>
+          <t>Es gibt Verantwortung. Keine vollständige Kontrolle.</t>
         </is>
       </c>
       <c r="P184" t="inlineStr"/>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>665</t>
+          <t>656</t>
         </is>
       </c>
       <c r="R184" t="inlineStr">
@@ -16620,36 +16778,36 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>20-F (Shot-Bereich 06:32–07:40)</t>
+          <t>20-E (Shot-Bereich 05:05–06:32)</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>20-F</t>
+          <t>20-E</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
+          <t>00:05:05:00</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
           <t>00:06:32:00</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>00:07:40:00</t>
-        </is>
-      </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>00:06:33:00</t>
+          <t>00:05:06:00</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>00:06:35:02</t>
+          <t>00:05:09:00</t>
         </is>
       </c>
       <c r="J185" t="n">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="K185" t="inlineStr">
         <is>
@@ -16673,13 +16831,13 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>Sind wir die Schöpfer?</t>
+          <t>Wer hat dann diese Welt erschaffen?</t>
         </is>
       </c>
       <c r="P185" t="inlineStr"/>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>669</t>
+          <t>660</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
@@ -16707,36 +16865,36 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>20-F (Shot-Bereich 06:32–07:40)</t>
+          <t>20-E (Shot-Bereich 05:05–06:32)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>20-F</t>
+          <t>20-E</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
+          <t>00:05:05:00</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
           <t>00:06:32:00</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>00:07:40:00</t>
-        </is>
-      </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>00:06:35:17</t>
+          <t>00:05:09:14</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>00:06:40:22</t>
+          <t>00:05:12:14</t>
         </is>
       </c>
       <c r="J186" t="n">
-        <v>5.2</v>
+        <v>3</v>
       </c>
       <c r="K186" t="inlineStr">
         <is>
@@ -16760,13 +16918,13 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>Wir sind Mitgestalter. Keiner von uns besitzt das Leben eines anderen.</t>
+          <t>Den ersten Ursprung kennen wir nicht.</t>
         </is>
       </c>
       <c r="P186" t="inlineStr"/>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>670</t>
+          <t>661</t>
         </is>
       </c>
       <c r="R186" t="inlineStr">
@@ -16794,36 +16952,36 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>20-F (Shot-Bereich 06:32–07:40)</t>
+          <t>20-E (Shot-Bereich 05:05–06:32)</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>20-F</t>
+          <t>20-E</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
+          <t>00:05:05:00</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
           <t>00:06:32:00</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>00:07:40:00</t>
-        </is>
-      </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>00:06:41:12</t>
+          <t>00:05:14:17</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>00:06:43:05</t>
+          <t>00:05:24:05</t>
         </is>
       </c>
       <c r="J187" t="n">
-        <v>1.7</v>
+        <v>9.5</v>
       </c>
       <c r="K187" t="inlineStr">
         <is>
@@ -16832,7 +16990,7 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
@@ -16847,13 +17005,13 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>Und das hier?</t>
+          <t>Aber die Welt, in der Menschen leben – ihre Häuser, Geschichten, Hoffnungen, ihre Wunden und ihre Möglichkeiten – formen sie miteinander.</t>
         </is>
       </c>
       <c r="P187" t="inlineStr"/>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>671</t>
+          <t>663</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -16881,36 +17039,36 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>20-F (Shot-Bereich 06:32–07:40)</t>
+          <t>20-E (Shot-Bereich 05:05–06:32)</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>20-F</t>
+          <t>20-E</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
+          <t>00:05:05:00</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
           <t>00:06:32:00</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>00:07:40:00</t>
-        </is>
-      </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>00:06:43:19</t>
+          <t>00:05:24:19</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>00:06:51:14</t>
+          <t>00:05:26:02</t>
         </is>
       </c>
       <c r="J188" t="n">
-        <v>7.8</v>
+        <v>1.3</v>
       </c>
       <c r="K188" t="inlineStr">
         <is>
@@ -16919,7 +17077,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M188" t="inlineStr">
@@ -16934,13 +17092,13 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>Eine Möglichkeit, Bedingungen für eine neue Welt zu schaffen. Das Leben darin wird seinen eigenen Weg finden.</t>
+          <t>Wir alle?</t>
         </is>
       </c>
       <c r="P188" t="inlineStr"/>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>664</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -16968,36 +17126,36 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+          <t>20-E (Shot-Bereich 05:05–06:32)</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>20-G</t>
+          <t>20-E</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>00:07:40:00</t>
+          <t>00:05:05:00</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>00:09:00:00</t>
+          <t>00:06:32:00</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>00:07:41:00</t>
+          <t>00:05:26:17</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>00:07:46:05</t>
+          <t>00:05:33:14</t>
         </is>
       </c>
       <c r="J189" t="n">
-        <v>5.2</v>
+        <v>6.9</v>
       </c>
       <c r="K189" t="inlineStr">
         <is>
@@ -17006,7 +17164,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M189" t="inlineStr">
@@ -17021,13 +17179,13 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>Wenn ich mich entscheide … weiß ich dann, was daraus wird?</t>
+          <t>Mit jedem Leben. Mit dem, was wir tun. Und mit dem, was wir anderen ermöglichen.</t>
         </is>
       </c>
       <c r="P189" t="inlineStr"/>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>676</t>
+          <t>665</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -17055,36 +17213,36 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+          <t>20-F (Shot-Bereich 06:32–07:40)</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>20-G</t>
+          <t>20-F</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
+          <t>00:06:32:00</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
           <t>00:07:40:00</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>00:09:00:00</t>
-        </is>
-      </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>00:07:46:19</t>
+          <t>00:06:33:00</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>00:07:47:14</t>
+          <t>00:06:35:02</t>
         </is>
       </c>
       <c r="J190" t="n">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -17093,7 +17251,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M190" t="inlineStr">
@@ -17108,13 +17266,13 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>Nein.</t>
+          <t>Sind wir die Schöpfer?</t>
         </is>
       </c>
       <c r="P190" t="inlineStr"/>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>677</t>
+          <t>669</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
@@ -17142,36 +17300,36 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+          <t>20-F (Shot-Bereich 06:32–07:40)</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>20-G</t>
+          <t>20-F</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
+          <t>00:06:32:00</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
           <t>00:07:40:00</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>00:09:00:00</t>
-        </is>
-      </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>00:07:48:05</t>
+          <t>00:06:35:17</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>00:07:50:19</t>
+          <t>00:06:40:22</t>
         </is>
       </c>
       <c r="J191" t="n">
-        <v>2.6</v>
+        <v>5.2</v>
       </c>
       <c r="K191" t="inlineStr">
         <is>
@@ -17180,7 +17338,7 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M191" t="inlineStr">
@@ -17195,13 +17353,13 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>Dann kann ich Fehler machen.</t>
+          <t>Wir sind Mitgestalter. Keiner von uns besitzt das Leben eines anderen.</t>
         </is>
       </c>
       <c r="P191" t="inlineStr"/>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>678</t>
+          <t>670</t>
         </is>
       </c>
       <c r="R191" t="inlineStr">
@@ -17229,36 +17387,36 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+          <t>20-F (Shot-Bereich 06:32–07:40)</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>20-G</t>
+          <t>20-F</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
+          <t>00:06:32:00</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
           <t>00:07:40:00</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>00:09:00:00</t>
-        </is>
-      </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>00:07:51:10</t>
+          <t>00:06:41:12</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>00:07:52:05</t>
+          <t>00:06:43:05</t>
         </is>
       </c>
       <c r="J192" t="n">
-        <v>0.8</v>
+        <v>1.7</v>
       </c>
       <c r="K192" t="inlineStr">
         <is>
@@ -17267,7 +17425,7 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M192" t="inlineStr">
@@ -17282,13 +17440,13 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>Ja.</t>
+          <t>Und das hier?</t>
         </is>
       </c>
       <c r="P192" t="inlineStr"/>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>679</t>
+          <t>671</t>
         </is>
       </c>
       <c r="R192" t="inlineStr">
@@ -17316,36 +17474,36 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+          <t>20-F (Shot-Bereich 06:32–07:40)</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>20-G</t>
+          <t>20-F</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
+          <t>00:06:32:00</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
           <t>00:07:40:00</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr">
-        <is>
-          <t>00:09:00:00</t>
-        </is>
-      </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>00:07:52:19</t>
+          <t>00:06:43:19</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>00:07:55:10</t>
+          <t>00:06:51:14</t>
         </is>
       </c>
       <c r="J193" t="n">
-        <v>2.6</v>
+        <v>7.8</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -17354,7 +17512,7 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>SPIELER-ECHO</t>
+          <t>STIMMEN</t>
         </is>
       </c>
       <c r="M193" t="inlineStr">
@@ -17369,13 +17527,13 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>Und trotzdem darf ich anfangen?</t>
+          <t>Eine Möglichkeit, Bedingungen für eine neue Welt zu schaffen. Das Leben darin wird seinen eigenen Weg finden.</t>
         </is>
       </c>
       <c r="P193" t="inlineStr"/>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>672</t>
         </is>
       </c>
       <c r="R193" t="inlineStr">
@@ -17423,16 +17581,16 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>00:07:56:00</t>
+          <t>00:07:41:00</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>00:07:58:14</t>
+          <t>00:07:46:05</t>
         </is>
       </c>
       <c r="J194" t="n">
-        <v>2.6</v>
+        <v>5.2</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -17441,7 +17599,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M194" t="inlineStr">
@@ -17456,13 +17614,13 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>Du darfst mitgestalten. Nicht herrschen.</t>
+          <t>Wenn ich mich entscheide … weiß ich dann, was daraus wird?</t>
         </is>
       </c>
       <c r="P194" t="inlineStr"/>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>681</t>
+          <t>676</t>
         </is>
       </c>
       <c r="R194" t="inlineStr">
@@ -17475,51 +17633,51 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>VO_C21_001</t>
+          <t>VO_C20_034</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>SUB_C21_001</t>
+          <t>SUB_C20_034</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>21-D (Shot-Bereich 02:25–03:10)</t>
+          <t>20-G (Shot-Bereich 07:40–09:00)</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>21-D</t>
+          <t>20-G</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>00:02:25:00</t>
+          <t>00:07:40:00</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>00:03:10:00</t>
+          <t>00:09:00:00</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>00:02:26:00</t>
+          <t>00:07:46:19</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>00:02:29:22</t>
+          <t>00:07:47:14</t>
         </is>
       </c>
       <c r="J195" t="n">
-        <v>3.9</v>
+        <v>0.8</v>
       </c>
       <c r="K195" t="inlineStr">
         <is>
@@ -17543,17 +17701,13 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>Wir wissen nicht, wer sie einmal sein werden.</t>
-        </is>
-      </c>
-      <c r="P195" t="inlineStr">
-        <is>
-          <t>fast unhörbar, nicht als verkündender Erzähler</t>
-        </is>
-      </c>
+          <t>Nein.</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr"/>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>699</t>
+          <t>677</t>
         </is>
       </c>
       <c r="R195" t="inlineStr">
@@ -17566,51 +17720,51 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>VO_C21_002</t>
+          <t>VO_C20_035</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>SUB_C21_002</t>
+          <t>SUB_C20_035</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>21-D (Shot-Bereich 02:25–03:10)</t>
+          <t>20-G (Shot-Bereich 07:40–09:00)</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>21-D</t>
+          <t>20-G</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>00:02:25:00</t>
+          <t>00:07:40:00</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>00:03:10:00</t>
+          <t>00:09:00:00</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>00:02:32:00</t>
+          <t>00:07:48:05</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>00:02:34:02</t>
+          <t>00:07:50:19</t>
         </is>
       </c>
       <c r="J196" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="K196" t="inlineStr">
         <is>
@@ -17619,7 +17773,7 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>STIMMEN</t>
+          <t>SPIELER-ECHO</t>
         </is>
       </c>
       <c r="M196" t="inlineStr">
@@ -17634,24 +17788,463 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>Das ist ihr Leben.</t>
+          <t>Dann kann ich Fehler machen.</t>
         </is>
       </c>
       <c r="P196" t="inlineStr"/>
       <c r="Q196" t="inlineStr">
         <is>
+          <t>678</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>Zeitcode vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="S196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>VO_C20_036</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>SUB_C20_036</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>20-G</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>00:07:40:00</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>00:09:00:00</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>00:07:51:10</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>00:07:52:05</t>
+        </is>
+      </c>
+      <c r="J197" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>STIMMEN</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>de-DE</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>Ja.</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr"/>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>679</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>Zeitcode vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>VO_C20_037</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>SUB_C20_037</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>20-G</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>00:07:40:00</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>00:09:00:00</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>00:07:52:19</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>00:07:55:10</t>
+        </is>
+      </c>
+      <c r="J198" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>SPIELER-ECHO</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>de-DE</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>Und trotzdem darf ich anfangen?</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr"/>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>680</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>Zeitcode vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="S198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>VO_C20_038</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>SUB_C20_038</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>20-G (Shot-Bereich 07:40–09:00)</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>20-G</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>00:07:40:00</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>00:09:00:00</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>00:07:56:00</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>00:07:58:14</t>
+        </is>
+      </c>
+      <c r="J199" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>STIMMEN</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>de-DE</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>Du darfst mitgestalten. Nicht herrschen.</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr"/>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>681</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>Zeitcode vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="S199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>VO_C21_001</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>SUB_C21_001</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>21-D (Shot-Bereich 02:25–03:10)</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>21-D</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>00:02:25:00</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>00:03:10:00</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>00:02:26:00</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>00:02:29:22</t>
+        </is>
+      </c>
+      <c r="J200" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>STIMMEN</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>de-DE</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>Wir wissen nicht, wer sie einmal sein werden.</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>fast unhörbar, nicht als verkündender Erzähler</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>699</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Zeitcode vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="S200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>VO_C21_002</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>SUB_C21_002</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>21-D (Shot-Bereich 02:25–03:10)</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>21-D</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>00:02:25:00</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>00:03:10:00</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>00:02:32:00</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>00:02:34:02</t>
+        </is>
+      </c>
+      <c r="J201" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>vorläufig/geschätzt</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>STIMMEN</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>de-DE</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>Das ist ihr Leben.</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr"/>
+      <c r="Q201" t="inlineStr">
+        <is>
           <t>701</t>
         </is>
       </c>
-      <c r="R196" t="inlineStr">
+      <c r="R201" t="inlineStr">
         <is>
           <t>Zeitcode vorläufig/geschätzt</t>
         </is>
       </c>
-      <c r="S196" t="inlineStr"/>
+      <c r="S201" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S196"/>
+  <autoFilter ref="A1:S201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>